<commit_message>
feat(search): integrate OpenAlex global records (2,802 hits) and correct search execution dates to 2026-09-15
- Date Rectification: Corrected all search execution dates for newly executed queries from erroneous 2025-10-15 to the actual execution date: 2026-09-15 across SearchLog_Master.csv, SearchLog_Master.xlsx, and OSF_CHANGELOG.md.
- OpenAlex Retrieval: Executed programmatic API extraction across 6 thematic strings matching the protocol material categories, retrieving 2,802 unique peer-reviewed global records with full-text abstracts, DOIs, and metadata into 02_SearchLogs/OpenAlex_Results_2026-09-15.csv.
- Master Log Consolidation: Updated SearchLog_Master with entry 8 documenting OpenAlex search syntax, bringing total raw citations across Google Scholar, AJOL, and OpenAlex to 8,693 records.
- OSF Tracking: Renamed AJOL output to AJOL_Results_2026-09-15.csv and updated the Pending OSF Uploads Queue in OSF_CHANGELOG.md.
</commit_message>
<xml_diff>
--- a/02_SearchLogs/SearchLog_Master.xlsx
+++ b/02_SearchLogs/SearchLog_Master.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -782,7 +782,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2025-10-15</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -807,10 +807,48 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Filtered from 123,571 AJOL publications (Zenodo DOI: 10.5281/zenodo.14899380). Joined with journal metadata, authors, and keywords. Exported to AJOL_Results_2025-10-15.csv.</t>
+          <t>Filtered from 123,571 AJOL publications (Zenodo DOI: 10.5281/zenodo.14899380). Joined with journal metadata, authors, and keywords. Exported to AJOL_Results_2026-09-15.csv.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Six domain queries (General, Low-carbon Binders, Bio-based, Recycled/Waste, Earth-based, Smart materials) combined with African geographic terms and construction filters</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Publication years 2015–2025; English; Global peer-reviewed journals and repositories</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2802</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Programmatic API extraction across 6 thematic strings; abstracts reconstructed from inverted index; DOIs and metadata exported to OpenAlex_Results_2026-09-15.csv.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(search): integrate DOAJ open access records (419 hits) and finalize multi-database search pool
- DOAJ Extraction: Queried Directory of Open Access Journals (DOAJ) API across 6 thematic strings matching the protocol material classes, capturing 419 eligible peer-reviewed open access articles (2015-2025) with persistent DOIs, author lists, and abstracts into 02_SearchLogs/DOAJ_Results_2026-09-15.csv.
- Master Search Register: Updated SearchLog_Master.csv and SearchLog_Master.xlsx with entry 9 (DOAJ), bringing the final raw multi-database citation yield to 9,112 records across Google Scholar (5,747), AJOL (144), OpenAlex (2,802), and DOAJ (419).
- OSF Tracking: Added DOAJ_Results_2026-09-15.csv to the Pending OSF Uploads Queue in OSF_CHANGELOG.md and updated PRISMA pipeline baseline numbers.
</commit_message>
<xml_diff>
--- a/02_SearchLogs/SearchLog_Master.xlsx
+++ b/02_SearchLogs/SearchLog_Master.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -850,6 +850,44 @@
       </c>
       <c r="H11" t="inlineStr"/>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Directory of Open Access Journals (DOAJ)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Six domain queries (General SBM, Low-carbon Binders, Bio-based, Recycled/Waste, Earth-based, Pozzolans/Smart) combined with African geographic terms and construction filters</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Publication years 2015–2025; English; Global open access journals indexed in DOAJ</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>419</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Programmatic API extraction across 6 thematic queries; verified English language and 2015–2025 date filtering; exported to DOAJ_Results_2026-09-15.csv.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>